<commit_message>
Preamble to matrix multiplication
</commit_message>
<xml_diff>
--- a/calculations/input/groupWprefixes.xlsx
+++ b/calculations/input/groupWprefixes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9964733-025F-489C-AE5B-34C183A13DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31C049E-1C29-4EAE-9FBA-9D1BF6F0C52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5B2A76A6-A912-46C2-946E-7449FD39B25B}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{5B2A76A6-A912-46C2-946E-7449FD39B25B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Groups</t>
   </si>
   <si>
-    <t>tfp</t>
-  </si>
-  <si>
     <t>gva</t>
   </si>
   <si>
@@ -56,9 +53,6 @@
     <t>l</t>
   </si>
   <si>
-    <t>z</t>
-  </si>
-  <si>
     <t>y</t>
   </si>
   <si>
@@ -77,9 +71,6 @@
     <t>W_g3</t>
   </si>
   <si>
-    <t>W²_g1</t>
-  </si>
-  <si>
     <t>W_g1W_g2</t>
   </si>
   <si>
@@ -101,33 +92,6 @@
     <t>W_d3</t>
   </si>
   <si>
-    <t>W²_d1</t>
-  </si>
-  <si>
-    <t>W²_d2</t>
-  </si>
-  <si>
-    <t>W²_d3</t>
-  </si>
-  <si>
-    <t>W³_d1</t>
-  </si>
-  <si>
-    <t>W³_d2</t>
-  </si>
-  <si>
-    <t>W³_d3</t>
-  </si>
-  <si>
-    <t>W⁴_d1</t>
-  </si>
-  <si>
-    <t>W⁴_d2</t>
-  </si>
-  <si>
-    <t>W⁴_d3</t>
-  </si>
-  <si>
     <t>W_g2W_g1</t>
   </si>
   <si>
@@ -135,6 +99,36 @@
   </si>
   <si>
     <t>W_g1W_g3</t>
+  </si>
+  <si>
+    <t>W^2_d1</t>
+  </si>
+  <si>
+    <t>W^2_d2</t>
+  </si>
+  <si>
+    <t>W^2_d3</t>
+  </si>
+  <si>
+    <t>W^3_d1</t>
+  </si>
+  <si>
+    <t>W^3_d2</t>
+  </si>
+  <si>
+    <t>W^3_d3</t>
+  </si>
+  <si>
+    <t>W^4_d1</t>
+  </si>
+  <si>
+    <t>W^4_d2</t>
+  </si>
+  <si>
+    <t>W^4_d3</t>
+  </si>
+  <si>
+    <t>W^2_g1</t>
   </si>
 </sst>
 </file>
@@ -523,602 +517,507 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A65B007-5B57-49B3-BF45-73B8C2F1F293}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="3" t="str">
+        <f t="shared" ref="B4:B13" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A4,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
+        <v>wg1</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" ref="C4:E4" si="1">_xlfn.TEXTJOIN("_", TRUE, $B4, C$2)</f>
+        <v>wg1_gva</v>
+      </c>
+      <c r="D4" t="str">
+        <f t="shared" si="1"/>
+        <v>wg1_capital</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="1"/>
+        <v>wg1_labour</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg2</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" ref="C5:E26" si="2">_xlfn.TEXTJOIN("_", TRUE, $B5, C$2)</f>
+        <v>wg2_gva</v>
+      </c>
+      <c r="D5" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2_capital</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2_labour</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="str">
-        <f>LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A4, "_", ""), "²", "2"), "³", "3"), "⁴", "4"))</f>
-        <v>wg1</v>
-      </c>
-      <c r="C4" t="str">
-        <f>_xlfn.TEXTJOIN("_", TRUE, $B4, C$2)</f>
-        <v>wg1_tfp</v>
-      </c>
-      <c r="D4" t="str">
-        <f t="shared" ref="D4:F4" si="0">_xlfn.TEXTJOIN("_", TRUE, $B4, D$2)</f>
-        <v>wg1_gva</v>
-      </c>
-      <c r="E4" t="str">
+      <c r="B6" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>wg1_capital</v>
-      </c>
-      <c r="F4" t="str">
+        <v>wg3</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3_gva</v>
+      </c>
+      <c r="D6" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3_capital</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3_labour</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>wg1_labour</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+        <v>w2g1</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="2"/>
+        <v>w2g1_gva</v>
+      </c>
+      <c r="D7" t="str">
+        <f t="shared" si="2"/>
+        <v>w2g1_capital</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="2"/>
+        <v>w2g1_labour</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3" t="str">
-        <f t="shared" ref="B5:B26" si="1">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A5, "_", ""), "²", "2"), "³", "3"), "⁴", "4"))</f>
-        <v>wg2</v>
-      </c>
-      <c r="C5" t="str">
-        <f t="shared" ref="C5:F26" si="2">_xlfn.TEXTJOIN("_", TRUE, $B5, C$2)</f>
-        <v>wg2_tfp</v>
-      </c>
-      <c r="D5" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2_gva</v>
-      </c>
-      <c r="E5" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2_capital</v>
-      </c>
-      <c r="F5" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2_labour</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg1wg2</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg2_gva</v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg2_capital</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg2_labour</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg3</v>
-      </c>
-      <c r="C6" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3_tfp</v>
-      </c>
-      <c r="D6" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3_gva</v>
-      </c>
-      <c r="E6" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3_capital</v>
-      </c>
-      <c r="F6" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3_labour</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="B9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg2wg3</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg3_gva</v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg3_capital</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg3_labour</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>w2g1</v>
-      </c>
-      <c r="C7" t="str">
-        <f t="shared" si="2"/>
-        <v>w2g1_tfp</v>
-      </c>
-      <c r="D7" t="str">
-        <f t="shared" si="2"/>
-        <v>w2g1_gva</v>
-      </c>
-      <c r="E7" t="str">
-        <f t="shared" si="2"/>
-        <v>w2g1_capital</v>
-      </c>
-      <c r="F7" t="str">
-        <f t="shared" si="2"/>
-        <v>w2g1_labour</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="B10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg3wg1</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg1_gva</v>
+      </c>
+      <c r="D10" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg1_capital</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg1_labour</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg2wg1</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg1_gva</v>
+      </c>
+      <c r="D11" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg1_capital</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="2"/>
+        <v>wg2wg1_labour</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg3wg2</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg2_gva</v>
+      </c>
+      <c r="D12" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg2_capital</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="2"/>
+        <v>wg3wg2_labour</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>wg1wg3</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg3_gva</v>
+      </c>
+      <c r="D13" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg3_capital</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="2"/>
+        <v>wg1wg3_labour</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg1wg2</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_tfp</v>
-      </c>
-      <c r="D8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_gva</v>
-      </c>
-      <c r="E8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_capital</v>
-      </c>
-      <c r="F8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_labour</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg2wg3</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg3_tfp</v>
-      </c>
-      <c r="D9" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg3_gva</v>
-      </c>
-      <c r="E9" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg3_capital</v>
-      </c>
-      <c r="F9" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg3_labour</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="B15" s="3" t="str">
+        <f t="shared" ref="B15:B26" si="3">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A15,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
+        <v>wd1</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="2"/>
+        <v>wd1_gva</v>
+      </c>
+      <c r="D15" t="str">
+        <f t="shared" si="2"/>
+        <v>wd1_capital</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="2"/>
+        <v>wd1_labour</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg3wg1</v>
-      </c>
-      <c r="C10" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg1_tfp</v>
-      </c>
-      <c r="D10" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg1_gva</v>
-      </c>
-      <c r="E10" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg1_capital</v>
-      </c>
-      <c r="F10" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg1_labour</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg2wg1</v>
-      </c>
-      <c r="C11" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg1_tfp</v>
-      </c>
-      <c r="D11" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg1_gva</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg1_capital</v>
-      </c>
-      <c r="F11" t="str">
-        <f t="shared" si="2"/>
-        <v>wg2wg1_labour</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg3wg2</v>
-      </c>
-      <c r="C12" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg2_tfp</v>
-      </c>
-      <c r="D12" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg2_gva</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg2_capital</v>
-      </c>
-      <c r="F12" t="str">
-        <f t="shared" si="2"/>
-        <v>wg3wg2_labour</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wg1wg3</v>
-      </c>
-      <c r="C13" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg3_tfp</v>
-      </c>
-      <c r="D13" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg3_gva</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg3_capital</v>
-      </c>
-      <c r="F13" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg3_labour</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>wd2</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="2"/>
+        <v>wd2_gva</v>
+      </c>
+      <c r="D16" t="str">
+        <f t="shared" si="2"/>
+        <v>wd2_capital</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="2"/>
+        <v>wd2_labour</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wd1</v>
-      </c>
-      <c r="C15" t="str">
-        <f t="shared" si="2"/>
-        <v>wd1_tfp</v>
-      </c>
-      <c r="D15" t="str">
-        <f t="shared" si="2"/>
-        <v>wd1_gva</v>
-      </c>
-      <c r="E15" t="str">
-        <f t="shared" si="2"/>
-        <v>wd1_capital</v>
-      </c>
-      <c r="F15" t="str">
-        <f t="shared" si="2"/>
-        <v>wd1_labour</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>wd2</v>
-      </c>
-      <c r="C16" t="str">
-        <f t="shared" si="2"/>
-        <v>wd2_tfp</v>
-      </c>
-      <c r="D16" t="str">
-        <f t="shared" si="2"/>
-        <v>wd2_gva</v>
-      </c>
-      <c r="E16" t="str">
-        <f t="shared" si="2"/>
-        <v>wd2_capital</v>
-      </c>
-      <c r="F16" t="str">
-        <f t="shared" si="2"/>
-        <v>wd2_labour</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="B17" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>wd3</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="2"/>
-        <v>wd3_tfp</v>
+        <v>wd3_gva</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="2"/>
-        <v>wd3_gva</v>
+        <v>wd3_capital</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="2"/>
-        <v>wd3_capital</v>
-      </c>
-      <c r="F17" t="str">
-        <f t="shared" si="2"/>
         <v>wd3_labour</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w2d1</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="2"/>
-        <v>w2d1_tfp</v>
+        <v>w2d1_gva</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="2"/>
-        <v>w2d1_gva</v>
+        <v>w2d1_capital</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="2"/>
-        <v>w2d1_capital</v>
-      </c>
-      <c r="F18" t="str">
-        <f t="shared" si="2"/>
         <v>w2d1_labour</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B19" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w2d2</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="2"/>
-        <v>w2d2_tfp</v>
+        <v>w2d2_gva</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="2"/>
-        <v>w2d2_gva</v>
+        <v>w2d2_capital</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="2"/>
-        <v>w2d2_capital</v>
-      </c>
-      <c r="F19" t="str">
-        <f t="shared" si="2"/>
         <v>w2d2_labour</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B20" si="4">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A20,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
         <v>w2d3</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="2"/>
-        <v>w2d3_tfp</v>
+        <v>w2d3_gva</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="2"/>
-        <v>w2d3_gva</v>
+        <v>w2d3_capital</v>
       </c>
       <c r="E20" t="str">
         <f t="shared" si="2"/>
-        <v>w2d3_capital</v>
-      </c>
-      <c r="F20" t="str">
-        <f t="shared" si="2"/>
         <v>w2d3_labour</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B21" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w3d1</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="2"/>
-        <v>w3d1_tfp</v>
+        <v>w3d1_gva</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="2"/>
-        <v>w3d1_gva</v>
+        <v>w3d1_capital</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="2"/>
-        <v>w3d1_capital</v>
-      </c>
-      <c r="F21" t="str">
-        <f t="shared" si="2"/>
         <v>w3d1_labour</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B22" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w3d2</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="2"/>
-        <v>w3d2_tfp</v>
+        <v>w3d2_gva</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="2"/>
-        <v>w3d2_gva</v>
+        <v>w3d2_capital</v>
       </c>
       <c r="E22" t="str">
         <f t="shared" si="2"/>
-        <v>w3d2_capital</v>
-      </c>
-      <c r="F22" t="str">
-        <f t="shared" si="2"/>
         <v>w3d2_labour</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w3d3</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="2"/>
-        <v>w3d3_tfp</v>
+        <v>w3d3_gva</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="2"/>
-        <v>w3d3_gva</v>
+        <v>w3d3_capital</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="2"/>
-        <v>w3d3_capital</v>
-      </c>
-      <c r="F23" t="str">
-        <f t="shared" si="2"/>
         <v>w3d3_labour</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B24" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w4d1</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="2"/>
-        <v>w4d1_tfp</v>
+        <v>w4d1_gva</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="2"/>
-        <v>w4d1_gva</v>
+        <v>w4d1_capital</v>
       </c>
       <c r="E24" t="str">
         <f t="shared" si="2"/>
-        <v>w4d1_capital</v>
-      </c>
-      <c r="F24" t="str">
-        <f t="shared" si="2"/>
         <v>w4d1_labour</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B25" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w4d2</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="2"/>
-        <v>w4d2_tfp</v>
+        <v>w4d2_gva</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="2"/>
-        <v>w4d2_gva</v>
+        <v>w4d2_capital</v>
       </c>
       <c r="E25" t="str">
         <f t="shared" si="2"/>
-        <v>w4d2_capital</v>
-      </c>
-      <c r="F25" t="str">
-        <f t="shared" si="2"/>
         <v>w4d2_labour</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B26" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>w4d3</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="2"/>
-        <v>w4d3_tfp</v>
+        <v>w4d3_gva</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="2"/>
-        <v>w4d3_gva</v>
+        <v>w4d3_capital</v>
       </c>
       <c r="E26" t="str">
-        <f t="shared" si="2"/>
-        <v>w4d3_capital</v>
-      </c>
-      <c r="F26" t="str">
         <f t="shared" si="2"/>
         <v>w4d3_labour</v>
       </c>

</xml_diff>

<commit_message>
Started implemetning W W^2 algorithm
</commit_message>
<xml_diff>
--- a/calculations/input/groupWprefixes.xlsx
+++ b/calculations/input/groupWprefixes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31C049E-1C29-4EAE-9FBA-9D1BF6F0C52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63278C1E-B135-4681-82DE-02021CF07396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{5B2A76A6-A912-46C2-946E-7449FD39B25B}"/>
   </bookViews>
@@ -71,9 +71,6 @@
     <t>W_g3</t>
   </si>
   <si>
-    <t>W_g1W_g2</t>
-  </si>
-  <si>
     <t>W_g2W_g3</t>
   </si>
   <si>
@@ -129,13 +126,16 @@
   </si>
   <si>
     <t>W^2_g1</t>
+  </si>
+  <si>
+    <t>W_{g1W_g2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,18 +146,31 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -172,15 +185,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -522,35 +536,36 @@
   <cols>
     <col min="1" max="1" width="13.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -558,19 +573,19 @@
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3" t="str">
+      <c r="B4" s="4" t="str">
         <f t="shared" ref="B4:B13" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A4,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
         <v>wg1</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" s="2" t="str">
         <f t="shared" ref="C4:E4" si="1">_xlfn.TEXTJOIN("_", TRUE, $B4, C$2)</f>
         <v>wg1_gva</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4" s="2" t="str">
         <f t="shared" si="1"/>
         <v>wg1_capital</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E4" s="2" t="str">
         <f t="shared" si="1"/>
         <v>wg1_labour</v>
       </c>
@@ -579,19 +594,19 @@
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="str">
+      <c r="B5" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg2</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" s="2" t="str">
         <f t="shared" ref="C5:E26" si="2">_xlfn.TEXTJOIN("_", TRUE, $B5, C$2)</f>
         <v>wg2_gva</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2_capital</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E5" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2_labour</v>
       </c>
@@ -600,424 +615,424 @@
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="str">
+      <c r="B6" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg3</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3_gva</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3_capital</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E6" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3_labour</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="3" t="str">
+        <v>28</v>
+      </c>
+      <c r="B7" s="4" t="str">
         <f t="shared" si="0"/>
         <v>w2g1</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2g1_gva</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2g1_capital</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E7" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2g1_labour</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="3" t="str">
+        <v>29</v>
+      </c>
+      <c r="B8" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>wg1wg2</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_gva</v>
-      </c>
-      <c r="D8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_capital</v>
-      </c>
-      <c r="E8" t="str">
-        <f t="shared" si="2"/>
-        <v>wg1wg2_labour</v>
+        <v>w{g1wg2</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>w{g1wg2_gva</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>w{g1wg2_capital</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>w{g1wg2_labour</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="3" t="str">
+        <v>10</v>
+      </c>
+      <c r="B9" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg2wg3</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C9" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg3_gva</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D9" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg3_capital</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E9" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg3_labour</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="3" t="str">
+        <v>11</v>
+      </c>
+      <c r="B10" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg3wg1</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C10" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg1_gva</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg1_capital</v>
       </c>
-      <c r="E10" t="str">
+      <c r="E10" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg1_labour</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="3" t="str">
+        <v>16</v>
+      </c>
+      <c r="B11" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg2wg1</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C11" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg1_gva</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg1_capital</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E11" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg2wg1_labour</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="3" t="str">
+        <v>17</v>
+      </c>
+      <c r="B12" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg3wg2</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg2_gva</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg2_capital</v>
       </c>
-      <c r="E12" t="str">
+      <c r="E12" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg3wg2_labour</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="3" t="str">
+        <v>18</v>
+      </c>
+      <c r="B13" s="4" t="str">
         <f t="shared" si="0"/>
         <v>wg1wg3</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg1wg3_gva</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D13" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg1wg3_capital</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E13" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wg1wg3_labour</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3"/>
+      <c r="A14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="str">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="str">
         <f t="shared" ref="B15:B26" si="3">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A15,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
         <v>wd1</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd1_gva</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D15" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd1_capital</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E15" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd1_labour</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="str">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="str">
         <f t="shared" si="3"/>
         <v>wd2</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd2_gva</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D16" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd2_capital</v>
       </c>
-      <c r="E16" t="str">
+      <c r="E16" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd2_labour</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="str">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="str">
         <f t="shared" si="3"/>
         <v>wd3</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C17" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd3_gva</v>
       </c>
-      <c r="D17" t="str">
+      <c r="D17" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd3_capital</v>
       </c>
-      <c r="E17" t="str">
+      <c r="E17" s="2" t="str">
         <f t="shared" si="2"/>
         <v>wd3_labour</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="3" t="str">
+        <v>19</v>
+      </c>
+      <c r="B18" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w2d1</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C18" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d1_gva</v>
       </c>
-      <c r="D18" t="str">
+      <c r="D18" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d1_capital</v>
       </c>
-      <c r="E18" t="str">
+      <c r="E18" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d1_labour</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="B19" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w2d2</v>
       </c>
-      <c r="C19" t="str">
+      <c r="C19" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d2_gva</v>
       </c>
-      <c r="D19" t="str">
+      <c r="D19" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d2_capital</v>
       </c>
-      <c r="E19" t="str">
+      <c r="E19" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d2_labour</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="3" t="str">
+        <v>21</v>
+      </c>
+      <c r="B20" s="4" t="str">
         <f t="shared" ref="B20" si="4">LOWER(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A20,"_",""),"²","2"),"³","3"),"⁴","4"),"^",""))</f>
         <v>w2d3</v>
       </c>
-      <c r="C20" t="str">
+      <c r="C20" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d3_gva</v>
       </c>
-      <c r="D20" t="str">
+      <c r="D20" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d3_capital</v>
       </c>
-      <c r="E20" t="str">
+      <c r="E20" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w2d3_labour</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="3" t="str">
+        <v>22</v>
+      </c>
+      <c r="B21" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w3d1</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C21" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d1_gva</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D21" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d1_capital</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E21" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d1_labour</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="3" t="str">
+        <v>23</v>
+      </c>
+      <c r="B22" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w3d2</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C22" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d2_gva</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D22" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d2_capital</v>
       </c>
-      <c r="E22" t="str">
+      <c r="E22" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d2_labour</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="3" t="str">
+        <v>24</v>
+      </c>
+      <c r="B23" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w3d3</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C23" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d3_gva</v>
       </c>
-      <c r="D23" t="str">
+      <c r="D23" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d3_capital</v>
       </c>
-      <c r="E23" t="str">
+      <c r="E23" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w3d3_labour</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="3" t="str">
+        <v>25</v>
+      </c>
+      <c r="B24" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w4d1</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C24" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d1_gva</v>
       </c>
-      <c r="D24" t="str">
+      <c r="D24" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d1_capital</v>
       </c>
-      <c r="E24" t="str">
+      <c r="E24" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d1_labour</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="3" t="str">
+        <v>26</v>
+      </c>
+      <c r="B25" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w4d2</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C25" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d2_gva</v>
       </c>
-      <c r="D25" t="str">
+      <c r="D25" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d2_capital</v>
       </c>
-      <c r="E25" t="str">
+      <c r="E25" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d2_labour</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="3" t="str">
+        <v>27</v>
+      </c>
+      <c r="B26" s="4" t="str">
         <f t="shared" si="3"/>
         <v>w4d3</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C26" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d3_gva</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D26" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d3_capital</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E26" s="2" t="str">
         <f t="shared" si="2"/>
         <v>w4d3_labour</v>
       </c>

</xml_diff>